<commit_message>
Knowledge log: White's Reality Check for Data Snooping
Added while discussing pivot filtering. Narrowing 7 pivots to the 4 that made
money is a choice among 128 subsets, and the best of 128 always looks good --
White's bootstrap tests the winner against the whole set of rules searched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/knowledge-log.xlsx
+++ b/docs/knowledge-log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Reading log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reading log'!$A$4:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reading log'!$A$4:$F$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -92,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -123,6 +123,36 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -490,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -548,22 +578,22 @@
       </c>
     </row>
     <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Exit &amp; trailing rules</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>Maximum Adverse Excursion — John Sweeney (Wiley, 1996)</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="16" t="inlineStr">
         <is>
           <t>Book / method</t>
         </is>
@@ -573,29 +603,29 @@
           <t>The canonical way to set a stop from data instead of a hunch: plot how far every trade went against you before it worked, and put the stop where only the losers reach. Exactly the analysis our trade records can't support yet.</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>https://nexusfi.com/wiki/trading-wiki/Maximum-Adverse-Excursion</t>
         </is>
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Exit &amp; trailing rules</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>MAE / MFE distributions</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>Article</t>
         </is>
@@ -605,29 +635,29 @@
           <t>Shorter, practical version of the same idea — plotting both excursions to tune stops and targets together. Good 10-minute read before we add MFE logging.</t>
         </is>
       </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="F6" s="19" t="inlineStr">
         <is>
           <t>https://www.luxalgo.com/library/concept/mae-mfe-distributions.md</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>Exit &amp; trailing rules</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>Chandelier Exit — Chuck LeBeau</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>Indicator</t>
         </is>
@@ -637,29 +667,29 @@
           <t>Trail a fixed number of ATRs below the highest high since entry, ratcheted so the stop never loosens. The borrowable idea: scale the trail to volatility rather than to a fixed R, so a quiet stock isn't given the same room as a violent one.</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>https://www.barchart.com/education/technical-indicators/chandelier-exit</t>
         </is>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Exit &amp; trailing rules</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Chandelier Stop — implementation notes</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>Article</t>
         </is>
@@ -669,29 +699,29 @@
           <t>Covers the detail most write-ups miss: the raw formula can actually lower a long stop when ATR expands without a new high, so a ratchet has to be added on top.</t>
         </is>
       </c>
-      <c r="F8" s="11" t="inlineStr">
+      <c r="F8" s="19" t="inlineStr">
         <is>
           <t>https://www.luxalgo.com/library/concept/chandelier-stop.md</t>
         </is>
       </c>
     </row>
     <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Exit &amp; trailing rules</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Trail on the underlying, not the option premium</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>Idea — untested</t>
         </is>
@@ -701,25 +731,25 @@
           <t>Our own idea, worth testing. The premium moves with delta, theta and vega at once, so a premium stop can fire on a volatility collapse even when the directional call was right. A stop on the stock, converted to a premium level, isolates what the strategy actually predicts.</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
+      <c r="F9" s="16" t="inlineStr"/>
     </row>
     <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>Strategy rules</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>MO1 Strategy Rulebook</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>Internal doc</t>
         </is>
@@ -729,29 +759,29 @@
           <t>Both strategies clause by clause, with worked examples and every released version.</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="F10" s="18" t="inlineStr">
         <is>
           <t>docs/strategy-rulebook.pdf</t>
         </is>
       </c>
     </row>
     <row r="11" ht="58" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>Exit &amp; trailing rules</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>Exit and Trailing Study</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>Internal doc</t>
         </is>
@@ -761,29 +791,29 @@
           <t>The analysis behind the proposed ladder change: profit concentration, the two defective rungs, and what the data cannot answer.</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>docs/exit-analysis.pdf</t>
         </is>
       </c>
     </row>
     <row r="12" ht="58" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>Exit &amp; trailing rules</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>The Probability of Backtest Overfitting — Bailey, Borwein, López de Prado &amp; Zhu (J. Computational Finance, 2016)</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>Paper</t>
         </is>
@@ -793,29 +823,29 @@
           <t>Directly answers the worry you raised — how do you know a rule is real and not fitted to the trades you already have. Gives a way to measure it: split the history into blocks and check whether the best in-sample rule still ranks in the top half out-of-sample. Worth reading before we commit to any tuned exit.</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="F12" s="19" t="inlineStr">
         <is>
           <t>https://papers.ssrn.com/abstract=2326253</t>
         </is>
       </c>
     </row>
     <row r="13" ht="58" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>Option skew &amp; pivot levels</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
         <is>
           <t>Stock Price Clustering on Option Expiration Dates — Ni, Pearson &amp; Poteshman (2005), Journal of Financial Economics</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>Paper</t>
         </is>
@@ -825,29 +855,29 @@
           <t>The academic evidence behind the desk’s whole OI idea: prices really do get pulled to strikes where option open interest is heaviest, because of how option dealers hedge. Read sections 1 and 5 for why a lopsided strike can hold price, and when (near expiry) that effect is strongest.</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="17" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jfineco.2004.08.005</t>
         </is>
       </c>
     </row>
     <row r="14" ht="58" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>Stop sizing across stocks</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Edge ratio (E-ratio) - Curtis Faith, Way of the Turtle (2007); IASG explainer "How to Measure the Edge of Your Trading Entry Signals" (2015)</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>Article</t>
         </is>
@@ -857,29 +887,29 @@
           <t>Answers how MAE/MFE can work across many different stocks: divide each trade's MAE and MFE by that stock's ATR at entry, then pool all trades. A random entry scores about 1.0, so it also shows whether our entry has an edge on its own, separately from the exit rule.</t>
         </is>
       </c>
-      <c r="F14" s="11" t="inlineStr">
+      <c r="F14" s="19" t="inlineStr">
         <is>
           <t>https://www.iasg.com/?p=596</t>
         </is>
       </c>
     </row>
     <row r="15" ht="58" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>Stop sizing across stocks</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>ATR and MAE/MFE Stops</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="16" t="inlineStr">
         <is>
           <t>Internal doc</t>
         </is>
@@ -889,29 +919,29 @@
           <t>Why the ₹550 stop leaves some stocks six times more room than others, how ATR and MAE/MFE work together across 58 stocks, and the database fields that would make the next study exact.</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="16" t="inlineStr">
         <is>
           <t>docs/atr-mae-stops.pdf</t>
         </is>
       </c>
     </row>
     <row r="16" ht="58" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>Pivot-point analysis</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>Support for Resistance: Technical Analysis and Intraday Exchange Rates — Carol Osler (2000), FRBNY Economic Policy Review</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>Paper</t>
         </is>
@@ -921,14 +951,174 @@
           <t>The rigorous version of what the new pivot panel lets you eyeball: Osler bootstrap-tests published support/resistance levels against randomly placed ones and finds trends stop at the real levels far more often — yet the publishers' own 'strength' ratings predicted nothing. Read it before concluding R3 is broken on 23 trades; the method section shows how to test a level against chance.</t>
         </is>
       </c>
-      <c r="F16" s="11" t="inlineStr">
+      <c r="F16" s="19" t="inlineStr">
         <is>
           <t>https://www.newyorkfed.org/medialibrary/media/research/epr/00v06n2/0007osle.pdf</t>
         </is>
       </c>
     </row>
+    <row r="17" ht="58" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Historical data storage</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Financial Data Structures — López de Prado, Advances in Financial Machine Learning, ch. 2 (Wiley 2018)</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Book / method</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Argues that fixed-interval bars are a poor way to sample a market — the clock ticks at the same rate whether 10 lots or 10,000 trade. Proposes sampling by tick count, volume or rupee value instead, which gets returns closer to IID. Read it before locking the archive to 1-minute bars: from raw ticks you can build any of these, from minute bars you never can.</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>https://mlfinpy.readthedocs.io/en/latest/FinancialDataStructure.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="58" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Historical data storage</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>NSE F&amp;O UDiFF Common Bhavcopy — derivatives reports</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>The free daily file carrying every F&amp;O contract's OHLC, volume and open interest, including everything since expired. A far better source for the EOD chain layer than a broker API. Note the legacy bhavcopy was discontinued 8 July 2024, so five years of history spans two formats.</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>https://www.nseindia.com/all-reports-derivatives</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Historical data storage</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Continuous Futures Contracts Methodology for Backtesting — Quantpedia</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>The same trap your Dhan script has, in its better-documented form. A series stitched from successive contracts carries jumps at every roll that are not P&amp;L, and backtests book them as if they were. Covers the roll triggers and the difference vs ratio adjustment choice — read it before deciding how to handle the ATM strike changing mid-trade.</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>https://quantpedia.com/continuous-futures-contracts-methodology-for-backtesting/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="58" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Historical data storage</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Big Data is Dead — Jordan Tigani (MotherDuck)</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Written by a founding engineer on Google BigQuery, arguing the industry sold scale nobody needed and that a laptop now outruns a data warehouse for most real workloads. Worth 15 minutes before you pick a database: your five years of OI is well under 1 GB, and the instinct to reach for a server-based system is the thing this essay talks people out of.</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>https://motherduck.com/blog/big-data-is-dead/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="58" customHeight="1">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>Pivot levels &amp; filtering</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>A Reality Check for Data Snooping - Halbert White (Econometrica 68(5), 2000)</t>
+        </is>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Direct hit on what we are about to do. You narrowed 7 pivots down to the 4 that made money; there are 128 such subsets and the best one always looks good. White's bootstrap tests the winner against the whole set of rules you searched, so you learn whether R2/P/S2/S3 is a real edge or the luckiest of 128 coin flips.</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="inlineStr">
+        <is>
+          <t>https://www.econometricsociety.org/publications/econometrica/2000/09/01/reality-check-data-snooping</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F16"/>
+  <autoFilter ref="A4:F21"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -942,6 +1132,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Knowledge log: ISIS-2 and the cost of slicing a result by subgroup
Logged alongside the setup separation. Being able to replay A, B and C apart
makes it easy to keep the best of the three, which is the same act ISIS-2 put
a name to.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/knowledge-log.xlsx
+++ b/docs/knowledge-log.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1210,6 +1210,38 @@
       <c r="F24" s="19" t="inlineStr">
         <is>
           <t>https://doi.org/10.1090/noti1105</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="inlineStr">
+        <is>
+          <t>Backtest engine: comparing setups</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>Subgroup analysis and the ISIS-2 astrological subgroups - ISIS-2 Collaborative Group (The Lancet, 1988), discussed in Sleight, 'Debate: Subgroup analyses in clinical trials' (Current Controlled Trials in Cardiovascular Medicine 1(1), 2000)</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Read this before picking the best of setups A, B and C. ISIS-2 proved aspirin saves lives after a heart attack, then split the result by star sign - and patients born under Gemini or Libra appeared to be harmed by it. The authors published that deliberately, to show what slicing one result into subgroups does. Three legs from one backtest is the same act: the best of the three will look better than the whole regardless of whether it is better, and the lesson is to decide which leg you believe in before you see its number, not after.</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/cvm-1-1-025</t>
         </is>
       </c>
     </row>

</xml_diff>